<commit_message>
Remove brand text and simplify UI
</commit_message>
<xml_diff>
--- a/dummy_attendees.xlsx
+++ b/dummy_attendees.xlsx
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -487,7 +487,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -504,7 +504,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -521,7 +521,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -538,7 +538,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -555,7 +555,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,7 +589,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -606,7 +606,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -640,7 +640,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -657,7 +657,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -674,7 +674,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -708,7 +708,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -742,7 +742,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -759,7 +759,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -776,7 +776,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -793,7 +793,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -810,7 +810,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -844,7 +844,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -861,7 +861,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -878,7 +878,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -895,7 +895,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -912,7 +912,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -929,7 +929,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -946,7 +946,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -963,7 +963,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -980,7 +980,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -997,7 +997,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1014,7 +1014,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1031,7 +1031,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1048,7 +1048,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1065,7 +1065,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1082,7 +1082,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1099,7 +1099,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1116,7 +1116,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1133,7 +1133,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1167,7 +1167,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1184,7 +1184,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1201,7 +1201,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1218,7 +1218,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1235,7 +1235,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1252,7 +1252,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1269,7 +1269,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1286,7 +1286,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1303,7 +1303,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1320,7 +1320,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1354,7 +1354,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1388,7 +1388,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1405,7 +1405,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1422,7 +1422,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1439,7 +1439,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1473,7 +1473,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1490,7 +1490,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1507,7 +1507,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1524,7 +1524,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1541,7 +1541,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1558,7 +1558,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1575,7 +1575,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1592,7 +1592,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1609,7 +1609,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1626,7 +1626,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1643,7 +1643,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1660,7 +1660,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1677,7 +1677,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1711,7 +1711,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1728,7 +1728,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1745,7 +1745,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1762,7 +1762,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1779,7 +1779,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -1796,7 +1796,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -1813,7 +1813,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -1830,7 +1830,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1864,7 +1864,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -1881,7 +1881,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -1898,7 +1898,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -1915,7 +1915,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -1932,7 +1932,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -1949,7 +1949,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1966,7 +1966,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -1983,7 +1983,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2000,7 +2000,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2017,7 +2017,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2034,7 +2034,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2051,7 +2051,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2085,7 +2085,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2102,7 +2102,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2119,7 +2119,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2136,7 +2136,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2153,7 +2153,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>롯데</t>
+          <t>회사 A</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">

</xml_diff>